<commit_message>
feat(demo): sembrar catálogo completo de 88 productos y lotes en la tienda demo con alertas FEFO reales
</commit_message>
<xml_diff>
--- a/inventario_ejemplo_kardo.xlsx
+++ b/inventario_ejemplo_kardo.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="459">
   <si>
     <t xml:space="preserve">SKU</t>
   </si>
@@ -147,7 +147,7 @@
     <t xml:space="preserve">2026-10-04</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-28</t>
+    <t xml:space="preserve">2026-10-27</t>
   </si>
   <si>
     <t xml:space="preserve">LAC-GLO-006</t>
@@ -264,657 +264,657 @@
     <t xml:space="preserve">2026-10-12</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-10-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAC-GLO-012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750101001128</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crema de Leche Gloria UHT 200ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CRM-2607A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-04-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-INC-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750102002019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gaseosa Inca Kola Sabor Original 500ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEBIDAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-IK-500-26A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-07-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-INC-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750102002026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gaseosa Inca Kola Sin Azucar 500ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-IK-ZERO-26B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-07-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-COC-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750102002033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gaseosa Coca Cola Sabor Original 500ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CC-500-26A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-COC-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750102002040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gaseosa Coca Cola Sin Azucar 500ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CC-ZERO-26B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-07-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-INC-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750102002057</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gaseosa Inca Kola Gordita Vidrio 750ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-IK-GOR-26C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-08-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-SPR-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750102002064</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gaseosa Sprite Lima-Limon 500ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-SP-500-26A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-07-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-SLU-007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750102002071</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agua Mineral San Luis Sin Gas 625ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-AG-SL-625</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-10-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-SMA-008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750102002088</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agua Mineral San Mateo con Gas 600ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-AG-SM-600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-SPO-009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750102002095</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bebida Rehidratante Sporade Frutos Rojos 500ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-SPO-FR-500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-GAT-010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750102002101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bebida Rehidratante Gatorade Cool Blue 500ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-GAT-CB-500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-CIF-011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750102002118</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bebida Citrica Cifrut Granadilla 500ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CIF-GR-500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-05-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-FRU-012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750102002125</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nectar Frugos del Valle Durazno 1L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-FRU-DZ-1L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIC-CUS-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750103003016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerveza Cusquena Dorada Botella 330ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LICORES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CUS-DOR-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIC-CUS-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750103003023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerveza Cusquena Negra Botella 330ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CUS-NEG-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIC-PIL-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750103003030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerveza Pilsen Callao Botella 630ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PIL-630-26A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIC-PIL-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750103003047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerveza Pilsen Callao Six Pack Lata 355ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PACK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PIL-SIX-26B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-08-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIC-CRI-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750103003054</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerveza Cristal Botella 650ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CRI-650-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIC-COR-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750103003061</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerveza Corona Extra Botella 355ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-COR-355-MEX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIC-STE-007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750103003078</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerveza Stella Artois Botella 330ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-STE-330-BEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-08-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIC-CAR-008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750103003085</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ron Cartavio Black Barrel 750ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-RON-CAR-BB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2028-10-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIC-GAL-009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750103003092</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pisco Cuatro Gallos Quebranta 700ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PIS-4G-QUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIC-JOH-010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750103003108</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whisky Johnnie Walker Red Label 750ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-JW-RED-750</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2029-07-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-LAY-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Papas Fritas Lays Clasicas 160g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNACKS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOLSA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-LAY-CLA-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-01-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-LAY-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Papas Fritas Lays Onduladas 150g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-LAY-OND-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-12-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-DOR-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tortillas de Maiz Doritos Mega Queso 150g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-DOR-QSO-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-01-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-CHI-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Snack de Maiz Chizitos Fiesta 140g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CHZ-FIE-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-12-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-PIQ-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piqueo Snax Familiar 200g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PIQ-SNX-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-01-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-CHI-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004068</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chifle Piurano Salado Karinto 120g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CHF-KAR-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-12-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-SUB-007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004075</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chocolate Sublime Clasico Tableta 30g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIDAD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-SUB-CLA-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-05-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-PRI-008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004082</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chocolate Princesa Crema de Mani 30g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PRI-CRE-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-04-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-TRI-009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004099</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chocolate Triangulo DOnofrio 30g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-TRI-DON-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-MOR-010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galletas Morochas Rellenas Paquete 6 unid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-MOR-PAQ-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-03-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-CAS-011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004112</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galletas Casino Menta Paquete 6 unid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CAS-MEN-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-03-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-PEP-012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004129</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galletas Dona Pepa Field Paquete 6 unid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-DNP-PAQ-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-SOD-013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004136</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galletas Soda Field Paquete 6 unid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-SOD-FIE-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNK-GOM-014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750104004143</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gomitas Ambrosoli Ositos Dulces 100g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-GOM-OSI-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMB-SFE-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750105005010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hot Dog de Pollo San Fernando 500g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMBUTIDOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-HD-POL-2610</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMB-SFE-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750105005027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jamonada Especial San Fernando 250g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-JAM-SFE-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMB-BRA-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750105005034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jamonada de Cerdo Braedt 200g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-JAM-BRA-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-11-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMB-OTT-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750105005041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tocino Ahumado Tiras Otto Kunz 180g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-TOC-OTT-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-11-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMB-SFE-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750105005058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chorizo Parrillero San Fernando 400g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CHO-PAR-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-11-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMB-PRE-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7750105005065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salchicha Huachana La Preferida 250g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-SAL-HUA-26</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-10-26</t>
   </si>
   <si>
-    <t xml:space="preserve">LAC-GLO-012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750101001128</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crema de Leche Gloria UHT 200ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-CRM-2607A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-04-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-INC-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750102002019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gaseosa Inca Kola Sabor Original 500ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEBIDAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-IK-500-26A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-07-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-INC-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750102002026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gaseosa Inca Kola Sin Azucar 500ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-IK-ZERO-26B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-07-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-COC-003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750102002033</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gaseosa Coca Cola Sabor Original 500ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-CC-500-26A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-COC-004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750102002040</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gaseosa Coca Cola Sin Azucar 500ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-CC-ZERO-26B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-07-29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-INC-005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750102002057</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gaseosa Inca Kola Gordita Vidrio 750ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-IK-GOR-26C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-08-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-SPR-006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750102002064</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gaseosa Sprite Lima-Limon 500ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-SP-500-26A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-07-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-SLU-007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750102002071</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agua Mineral San Luis Sin Gas 625ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-AG-SL-625</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-10-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-SMA-008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750102002088</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agua Mineral San Mateo con Gas 600ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-AG-SM-600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-SPO-009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750102002095</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bebida Rehidratante Sporade Frutos Rojos 500ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-SPO-FR-500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-GAT-010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750102002101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bebida Rehidratante Gatorade Cool Blue 500ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-GAT-CB-500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-CIF-011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750102002118</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bebida Citrica Cifrut Granadilla 500ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-CIF-GR-500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-05-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-FRU-012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750102002125</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nectar Frugos del Valle Durazno 1L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-FRU-DZ-1L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIC-CUS-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750103003016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cerveza Cusquena Dorada Botella 330ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LICORES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-CUS-DOR-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIC-CUS-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750103003023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cerveza Cusquena Negra Botella 330ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-CUS-NEG-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIC-PIL-003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750103003030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cerveza Pilsen Callao Botella 630ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-PIL-630-26A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIC-PIL-004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750103003047</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cerveza Pilsen Callao Six Pack Lata 355ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PACK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-PIL-SIX-26B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-08-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIC-CRI-005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750103003054</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cerveza Cristal Botella 650ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-CRI-650-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIC-COR-006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750103003061</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cerveza Corona Extra Botella 355ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-COR-355-MEX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIC-STE-007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750103003078</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cerveza Stella Artois Botella 330ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-STE-330-BEL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-08-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-08-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIC-CAR-008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750103003085</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ron Cartavio Black Barrel 750ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-RON-CAR-BB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-07-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2028-10-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIC-GAL-009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750103003092</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pisco Cuatro Gallos Quebranta 700ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-PIS-4G-QUE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIC-JOH-010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750103003108</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Whisky Johnnie Walker Red Label 750ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-JW-RED-750</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2029-07-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-LAY-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Papas Fritas Lays Clasicas 160g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNACKS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOLSA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-LAY-CLA-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-01-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-LAY-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Papas Fritas Lays Onduladas 150g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-LAY-OND-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-12-31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-DOR-003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004037</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tortillas de Maiz Doritos Mega Queso 150g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-DOR-QSO-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-01-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-CHI-004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004044</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Snack de Maiz Chizitos Fiesta 140g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-CHZ-FIE-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-12-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-PIQ-005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004051</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Piqueo Snax Familiar 200g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-PIQ-SNX-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-01-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-CHI-006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004068</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chifle Piurano Salado Karinto 120g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-CHF-KAR-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-12-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-SUB-007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004075</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chocolate Sublime Clasico Tableta 30g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIDAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-SUB-CLA-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-05-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-PRI-008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004082</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chocolate Princesa Crema de Mani 30g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-PRI-CRE-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-04-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-TRI-009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004099</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chocolate Triangulo DOnofrio 30g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-TRI-DON-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-MOR-010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004105</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Galletas Morochas Rellenas Paquete 6 unid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-MOR-PAQ-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-03-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-CAS-011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004112</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Galletas Casino Menta Paquete 6 unid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-CAS-MEN-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-03-31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-PEP-012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004129</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Galletas Dona Pepa Field Paquete 6 unid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-DNP-PAQ-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-SOD-013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004136</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Galletas Soda Field Paquete 6 unid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-SOD-FIE-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNK-GOM-014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750104004143</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gomitas Ambrosoli Ositos Dulces 100g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-GOM-OSI-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMB-SFE-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750105005010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hot Dog de Pollo San Fernando 500g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMBUTIDOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-HD-POL-2610</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMB-SFE-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750105005027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jamonada Especial San Fernando 250g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-JAM-SFE-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMB-BRA-003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750105005034</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jamonada de Cerdo Braedt 200g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-JAM-BRA-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-11-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMB-OTT-004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750105005041</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tocino Ahumado Tiras Otto Kunz 180g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-TOC-OTT-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-11-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMB-SFE-005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750105005058</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chorizo Parrillero San Fernando 400g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-CHO-PAR-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-11-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMB-PRE-006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7750105005065</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Salchicha Huachana La Preferida 250g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-SAL-HUA-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-27</t>
-  </si>
-  <si>
     <t xml:space="preserve">EMB-OTT-007</t>
   </si>
   <si>
@@ -978,6 +978,9 @@
     <t xml:space="preserve">2026-10-15</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-10-25</t>
+  </si>
+  <si>
     <t xml:space="preserve">PAN-BIM-003</t>
   </si>
   <si>
@@ -1065,7 +1068,7 @@
     <t xml:space="preserve">2026-10-18</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-25</t>
+    <t xml:space="preserve">2026-10-23</t>
   </si>
   <si>
     <t xml:space="preserve">ABA-COS-001</t>
@@ -3512,7 +3515,7 @@
         <v>320</v>
       </c>
       <c r="J59" t="s">
-        <v>299</v>
+        <v>321</v>
       </c>
       <c r="K59" t="n">
         <v>20</v>
@@ -3520,13 +3523,13 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B60" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C60" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D60" t="s">
         <v>313</v>
@@ -3541,13 +3544,13 @@
         <v>10.50</v>
       </c>
       <c r="H60" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="I60" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J60" t="s">
-        <v>44</v>
+        <v>299</v>
       </c>
       <c r="K60" t="n">
         <v>18</v>
@@ -3555,13 +3558,13 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B61" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C61" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D61" t="s">
         <v>313</v>
@@ -3576,13 +3579,13 @@
         <v>5.80</v>
       </c>
       <c r="H61" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="I61" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="J61" t="s">
-        <v>272</v>
+        <v>44</v>
       </c>
       <c r="K61" t="n">
         <v>24</v>
@@ -3590,13 +3593,13 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B62" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C62" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D62" t="s">
         <v>313</v>
@@ -3611,7 +3614,7 @@
         <v>5.90</v>
       </c>
       <c r="H62" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="I62" t="s">
         <v>315</v>
@@ -3625,13 +3628,13 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B63" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C63" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D63" t="s">
         <v>313</v>
@@ -3646,13 +3649,13 @@
         <v>4.00</v>
       </c>
       <c r="H63" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="I63" t="s">
         <v>114</v>
       </c>
       <c r="J63" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K63" t="n">
         <v>30</v>
@@ -3660,13 +3663,13 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B64" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C64" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D64" t="s">
         <v>313</v>
@@ -3681,13 +3684,13 @@
         <v>5.50</v>
       </c>
       <c r="H64" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="I64" t="s">
         <v>94</v>
       </c>
       <c r="J64" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="K64" t="n">
         <v>30</v>
@@ -3695,13 +3698,13 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B65" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C65" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D65" t="s">
         <v>313</v>
@@ -3716,13 +3719,13 @@
         <v>4.50</v>
       </c>
       <c r="H65" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="I65" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J65" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K65" t="n">
         <v>20</v>
@@ -3730,16 +3733,16 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B66" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C66" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D66" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E66" t="s">
         <v>201</v>
@@ -3751,7 +3754,7 @@
         <v>5.30</v>
       </c>
       <c r="H66" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="I66" t="s">
         <v>63</v>
@@ -3765,16 +3768,16 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B67" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C67" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D67" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E67" t="s">
         <v>201</v>
@@ -3786,7 +3789,7 @@
         <v>5.90</v>
       </c>
       <c r="H67" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="I67" t="s">
         <v>30</v>
@@ -3800,16 +3803,16 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B68" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C68" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D68" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E68" t="s">
         <v>41</v>
@@ -3821,7 +3824,7 @@
         <v>10.90</v>
       </c>
       <c r="H68" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="I68" t="s">
         <v>17</v>
@@ -3835,16 +3838,16 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B69" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C69" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D69" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E69" t="s">
         <v>41</v>
@@ -3856,13 +3859,13 @@
         <v>29.90</v>
       </c>
       <c r="H69" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="I69" t="s">
         <v>184</v>
       </c>
       <c r="J69" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K69" t="n">
         <v>20</v>
@@ -3870,16 +3873,16 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B70" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C70" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D70" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E70" t="s">
         <v>61</v>
@@ -3891,13 +3894,13 @@
         <v>3.20</v>
       </c>
       <c r="H70" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="I70" t="s">
         <v>23</v>
       </c>
       <c r="J70" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K70" t="n">
         <v>80</v>
@@ -3905,16 +3908,16 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B71" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C71" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D71" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E71" t="s">
         <v>61</v>
@@ -3926,13 +3929,13 @@
         <v>2.80</v>
       </c>
       <c r="H71" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="I71" t="s">
         <v>63</v>
       </c>
       <c r="J71" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K71" t="n">
         <v>60</v>
@@ -3940,16 +3943,16 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B72" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C72" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D72" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E72" t="s">
         <v>15</v>
@@ -3961,7 +3964,7 @@
         <v>6.50</v>
       </c>
       <c r="H72" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="I72" t="s">
         <v>184</v>
@@ -3975,16 +3978,16 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B73" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C73" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D73" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E73" t="s">
         <v>15</v>
@@ -3996,10 +3999,10 @@
         <v>7.80</v>
       </c>
       <c r="H73" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="I73" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J73" t="s">
         <v>185</v>
@@ -4010,19 +4013,19 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B74" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C74" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D74" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E74" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F74" t="n">
         <v>6.40</v>
@@ -4031,7 +4034,7 @@
         <v>8.90</v>
       </c>
       <c r="H74" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="I74" t="s">
         <v>36</v>
@@ -4045,19 +4048,19 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B75" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C75" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D75" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E75" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F75" t="n">
         <v>4.20</v>
@@ -4066,7 +4069,7 @@
         <v>5.90</v>
       </c>
       <c r="H75" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="I75" t="s">
         <v>30</v>
@@ -4080,19 +4083,19 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B76" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C76" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D76" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E76" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F76" t="n">
         <v>6.80</v>
@@ -4101,7 +4104,7 @@
         <v>9.50</v>
       </c>
       <c r="H76" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="I76" t="s">
         <v>94</v>
@@ -4115,19 +4118,19 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B77" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C77" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D77" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E77" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F77" t="n">
         <v>12.50</v>
@@ -4136,13 +4139,13 @@
         <v>16.90</v>
       </c>
       <c r="H77" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="I77" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J77" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K77" t="n">
         <v>30</v>
@@ -4150,16 +4153,16 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B78" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C78" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D78" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E78" t="s">
         <v>163</v>
@@ -4171,7 +4174,7 @@
         <v>7.50</v>
       </c>
       <c r="H78" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="I78" t="s">
         <v>30</v>
@@ -4185,16 +4188,16 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B79" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C79" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D79" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E79" t="s">
         <v>163</v>
@@ -4206,7 +4209,7 @@
         <v>8.50</v>
       </c>
       <c r="H79" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="I79" t="s">
         <v>63</v>
@@ -4220,16 +4223,16 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B80" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C80" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D80" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E80" t="s">
         <v>163</v>
@@ -4241,7 +4244,7 @@
         <v>6.80</v>
       </c>
       <c r="H80" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="I80" t="s">
         <v>94</v>
@@ -4255,16 +4258,16 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B81" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C81" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D81" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E81" t="s">
         <v>233</v>
@@ -4276,7 +4279,7 @@
         <v>4.50</v>
       </c>
       <c r="H81" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="I81" t="s">
         <v>17</v>
@@ -4290,16 +4293,16 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B82" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C82" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D82" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E82" t="s">
         <v>233</v>
@@ -4311,7 +4314,7 @@
         <v>4.00</v>
       </c>
       <c r="H82" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="I82" t="s">
         <v>178</v>
@@ -4325,16 +4328,16 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B83" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C83" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D83" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E83" t="s">
         <v>41</v>
@@ -4346,10 +4349,10 @@
         <v>14.90</v>
       </c>
       <c r="H83" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="I83" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="J83" t="s">
         <v>185</v>
@@ -4360,19 +4363,19 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B84" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C84" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="D84" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E84" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F84" t="n">
         <v>3.50</v>
@@ -4381,7 +4384,7 @@
         <v>5.00</v>
       </c>
       <c r="H84" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="I84" t="s">
         <v>17</v>
@@ -4395,16 +4398,16 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B85" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C85" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D85" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E85" t="s">
         <v>41</v>
@@ -4416,7 +4419,7 @@
         <v>4.50</v>
       </c>
       <c r="H85" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="I85" t="s">
         <v>94</v>
@@ -4430,16 +4433,16 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B86" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C86" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D86" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E86" t="s">
         <v>68</v>
@@ -4451,13 +4454,13 @@
         <v>5.00</v>
       </c>
       <c r="H86" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="I86" t="s">
         <v>63</v>
       </c>
       <c r="J86" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K86" t="n">
         <v>36</v>
@@ -4465,16 +4468,16 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B87" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C87" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D87" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E87" t="s">
         <v>41</v>
@@ -4486,13 +4489,13 @@
         <v>5.90</v>
       </c>
       <c r="H87" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="I87" t="s">
         <v>36</v>
       </c>
       <c r="J87" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K87" t="n">
         <v>36</v>
@@ -4500,16 +4503,16 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B88" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C88" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D88" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E88" t="s">
         <v>201</v>
@@ -4521,13 +4524,13 @@
         <v>9.20</v>
       </c>
       <c r="H88" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="I88" t="s">
         <v>30</v>
       </c>
       <c r="J88" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K88" t="n">
         <v>30</v>
@@ -4535,16 +4538,16 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B89" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C89" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D89" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E89" t="s">
         <v>41</v>
@@ -4556,13 +4559,13 @@
         <v>7.20</v>
       </c>
       <c r="H89" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="I89" t="s">
         <v>94</v>
       </c>
       <c r="J89" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K89" t="n">
         <v>30</v>

</xml_diff>